<commit_message>
Aerodrome pack: per-item guidance + sub-checklists (81/81 guidance, 41 sub-checklists), EASA ADR references with private-aerodrome scope note; inspector comment box always visible (incl. reason for N/A); SubChecklist column in template/converter
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packs/_TEMPLATE_checklist.xlsx
+++ b/packs/_TEMPLATE_checklist.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -443,9 +443,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -492,6 +490,13 @@
       <c r="A9" t="inlineStr">
         <is>
           <t>6) อัปเดตปีถัดไป: คัดลอกทั้งโฟลเดอร์เป็น &lt;version ใหม่&gt; แก้ checklist แล้ว build — รอบตรวจเก่าไม่ถูกกระทบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>7) SubChecklist = รายการตรวจย่อยของข้อนั้น (สิ่งที่ต้องดูว่ามี/ไม่มี) — 1 บรรทัดต่อ 1 หัวข้อ (หรือคั่นด้วย | ) จะกลายเป็นช่องติ๊กย่อยในแอป</t>
         </is>
       </c>
     </row>
@@ -506,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -526,6 +531,7 @@
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
     <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -614,6 +620,11 @@
           <t>Dual</t>
         </is>
       </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>SubChecklist</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -646,7 +657,6 @@
           <t>การควบคุมการจ้างช่วง</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>1</t>
@@ -657,7 +667,6 @@
           <t>Contract documentation</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>(ตัวอย่าง) A written contract exists for each contracted activity</t>
@@ -673,7 +682,6 @@
           <t>ORA.GEN.205</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>แฟ้มสัญญา</t>

</xml_diff>